<commit_message>
Datos embebidos en la pagina (sin dependencia externa), plantilla para nuevas redes y conversor con argumentos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/red-pot-kennedy-visor.xlsx
+++ b/datos/red-pot-kennedy-visor.xlsx
@@ -10,13 +10,14 @@
     <sheet sheetId="4" name="NODOS" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="ARISTAS" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="CONTROL" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="RED" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1696" uniqueCount="1156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1718" uniqueCount="1178">
   <si>
     <t>RED POT KENNEDY - DATOS DEL VISOR 3D</t>
   </si>
@@ -3484,6 +3485,72 @@
   </si>
   <si>
     <t>Total aristas</t>
+  </si>
+  <si>
+    <t>Clave</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>titulo</t>
+  </si>
+  <si>
+    <t>Red Territorial de Kennedy (POT) — Sistema Socioecológico</t>
+  </si>
+  <si>
+    <t>marca</t>
+  </si>
+  <si>
+    <t>RED TERRITORIAL DE KENNEDY (POT)</t>
+  </si>
+  <si>
+    <t>faq1_pregunta</t>
+  </si>
+  <si>
+    <t>¿Qué significan las relaciones entre nodos?</t>
+  </si>
+  <si>
+    <t>faq1_respuesta</t>
+  </si>
+  <si>
+    <t>Cada enlace es una relación territorial con justificación causal: articulación funcional, presión ecológica, fragmentación, encadenamiento económico, desplazamiento, soporte ecosistémico, gestión institucional o gobernanza. Se basan en el POT (Decreto 555 de 2021) y en evidencia local de Kennedy.</t>
+  </si>
+  <si>
+    <t>faq2_pregunta</t>
+  </si>
+  <si>
+    <t>¿Por qué la infraestructura presiona los humedales?</t>
+  </si>
+  <si>
+    <t>faq2_respuesta</t>
+  </si>
+  <si>
+    <t>Corabastos, la Av. Ciudad de Cali y el sellamiento del suelo externalizan costos (ruido, lixiviados, escorrentía) sobre El Burro, La Vaca y Techo, que el POT trata como polígonos aislados.</t>
+  </si>
+  <si>
+    <t>faq3_pregunta</t>
+  </si>
+  <si>
+    <t>¿Qué dice el POT y qué ocurre en el territorio?</t>
+  </si>
+  <si>
+    <t>faq3_respuesta</t>
+  </si>
+  <si>
+    <t>Cada relación contrasta la intención declarada por la norma con su efecto operativo real; las hipótesis se formulan con base en el Decreto 555 y en la evidencia territorial de cada conexión.</t>
+  </si>
+  <si>
+    <t>faq4_pregunta</t>
+  </si>
+  <si>
+    <t>¿Qué tensiones son críticas?</t>
+  </si>
+  <si>
+    <t>faq4_respuesta</t>
+  </si>
+  <si>
+    <t>Las de nivel crítico: la Av. Ciudad de Cali partiendo El Burro, los vertimientos de Corabastos sobre La Vaca, la remoción de arbolado hub y el ruido sobre la fauna endémica. Filtra por tipo de relación para verlas en la red.</t>
   </si>
 </sst>
 </file>
@@ -10153,4 +10220,107 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>1156</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1160</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1164</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1169</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>1172</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>1176</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1177</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Corrige coordenadas (proyeccion UTM exacta) y el boton Giro 3D
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/red-pot-kennedy-visor.xlsx
+++ b/datos/red-pot-kennedy-visor.xlsx
@@ -4096,7 +4096,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4295,7 +4295,7 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4466,7 +4466,7 @@
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4570,10 +4570,10 @@
         <v>1</v>
       </c>
       <c r="M2">
-        <v>4.656</v>
+        <v>4.66159</v>
       </c>
       <c r="N2">
-        <v>-74.14</v>
+        <v>-74.13137</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -4614,10 +4614,10 @@
         <v>1</v>
       </c>
       <c r="M3">
-        <v>4.63</v>
+        <v>4.63433</v>
       </c>
       <c r="N3">
-        <v>-74.157</v>
+        <v>-74.15546</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -4658,10 +4658,10 @@
         <v>1</v>
       </c>
       <c r="M4">
-        <v>4.615</v>
+        <v>4.61862</v>
       </c>
       <c r="N4">
-        <v>-74.174</v>
+        <v>-74.17954</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -4702,10 +4702,10 @@
         <v>1</v>
       </c>
       <c r="M5">
-        <v>4.6255</v>
+        <v>4.62962</v>
       </c>
       <c r="N5">
-        <v>-74.16</v>
+        <v>-74.15972</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -4746,10 +4746,10 @@
         <v>1</v>
       </c>
       <c r="M6">
-        <v>4.636</v>
+        <v>4.64062</v>
       </c>
       <c r="N6">
-        <v>-74.153</v>
+        <v>-74.14979</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -4790,10 +4790,10 @@
         <v>1</v>
       </c>
       <c r="M7">
-        <v>4.6249</v>
+        <v>4.62899</v>
       </c>
       <c r="N7">
-        <v>-74.162</v>
+        <v>-74.16255</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -4834,10 +4834,10 @@
         <v>1</v>
       </c>
       <c r="M8">
-        <v>4.6419</v>
+        <v>4.64681</v>
       </c>
       <c r="N8">
-        <v>-74.1478</v>
+        <v>-74.14243</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -4878,10 +4878,10 @@
         <v>1</v>
       </c>
       <c r="M9">
-        <v>4.6262</v>
+        <v>4.63034</v>
       </c>
       <c r="N9">
-        <v>-74.1514</v>
+        <v>-74.14754</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -4922,10 +4922,10 @@
         <v>1</v>
       </c>
       <c r="M10">
-        <v>4.612</v>
+        <v>4.61548</v>
       </c>
       <c r="N10">
-        <v>-74.176</v>
+        <v>-74.18238</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -4966,10 +4966,10 @@
         <v>1</v>
       </c>
       <c r="M11">
-        <v>4.63</v>
+        <v>4.63432</v>
       </c>
       <c r="N11">
-        <v>-74.15</v>
+        <v>-74.14556</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -5010,10 +5010,10 @@
         <v>1</v>
       </c>
       <c r="M12">
-        <v>4.633</v>
+        <v>4.63746</v>
       </c>
       <c r="N12">
-        <v>-74.144</v>
+        <v>-74.13706</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -5054,10 +5054,10 @@
         <v>1</v>
       </c>
       <c r="M13">
-        <v>4.635</v>
+        <v>4.63958</v>
       </c>
       <c r="N13">
-        <v>-74.1545</v>
+        <v>-74.15192</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -5098,10 +5098,10 @@
         <v>1</v>
       </c>
       <c r="M14">
-        <v>4.633</v>
+        <v>4.63745</v>
       </c>
       <c r="N14">
-        <v>-74.138</v>
+        <v>-74.12857</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -5142,10 +5142,10 @@
         <v>1</v>
       </c>
       <c r="M15">
-        <v>4.629</v>
+        <v>4.63329</v>
       </c>
       <c r="N15">
-        <v>-74.159</v>
+        <v>-74.1583</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -5186,10 +5186,10 @@
         <v>1</v>
       </c>
       <c r="M16">
-        <v>4.614</v>
+        <v>4.61757</v>
       </c>
       <c r="N16">
-        <v>-74.17</v>
+        <v>-74.17388</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
@@ -5230,10 +5230,10 @@
         <v>1</v>
       </c>
       <c r="M17">
-        <v>4.6225</v>
+        <v>4.62647</v>
       </c>
       <c r="N17">
-        <v>-74.159</v>
+        <v>-74.1583</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -5274,10 +5274,10 @@
         <v>1</v>
       </c>
       <c r="M18">
-        <v>4.64</v>
+        <v>4.6448</v>
       </c>
       <c r="N18">
-        <v>-74.14</v>
+        <v>-74.13139</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
@@ -5318,10 +5318,10 @@
         <v>1</v>
       </c>
       <c r="M19">
-        <v>4.621</v>
+        <v>4.62489</v>
       </c>
       <c r="N19">
-        <v>-74.154</v>
+        <v>-74.15123</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
@@ -5362,10 +5362,10 @@
         <v>1</v>
       </c>
       <c r="M20">
-        <v>4.623</v>
+        <v>4.62697</v>
       </c>
       <c r="N20">
-        <v>-74.148</v>
+        <v>-74.14273</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
@@ -5406,10 +5406,10 @@
         <v>1</v>
       </c>
       <c r="M21">
-        <v>4.6335</v>
+        <v>4.638</v>
       </c>
       <c r="N21">
-        <v>-74.155</v>
+        <v>-74.15263</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -5450,10 +5450,10 @@
         <v>1</v>
       </c>
       <c r="M22">
-        <v>4.6365</v>
+        <v>4.64115</v>
       </c>
       <c r="N22">
-        <v>-74.152</v>
+        <v>-74.14838</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -5494,10 +5494,10 @@
         <v>1</v>
       </c>
       <c r="M23">
-        <v>4.637</v>
+        <v>4.64167</v>
       </c>
       <c r="N23">
-        <v>-74.154</v>
+        <v>-74.15121</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
@@ -5538,10 +5538,10 @@
         <v>1</v>
       </c>
       <c r="M24">
-        <v>4.626</v>
+        <v>4.63014</v>
       </c>
       <c r="N24">
-        <v>-74.156</v>
+        <v>-74.15405</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
@@ -5582,10 +5582,10 @@
         <v>1</v>
       </c>
       <c r="M25">
-        <v>4.6355</v>
+        <v>4.6401</v>
       </c>
       <c r="N25">
-        <v>-74.1535</v>
+        <v>-74.1505</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
@@ -5626,10 +5626,10 @@
         <v>1</v>
       </c>
       <c r="M26">
-        <v>4.6345</v>
+        <v>4.63904</v>
       </c>
       <c r="N26">
-        <v>-74.15</v>
+        <v>-74.14555</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
@@ -5670,10 +5670,10 @@
         <v>1</v>
       </c>
       <c r="M27">
-        <v>4.6245</v>
+        <v>4.62857</v>
       </c>
       <c r="N27">
-        <v>-74.161</v>
+        <v>-74.16113</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
@@ -5714,10 +5714,10 @@
         <v>1</v>
       </c>
       <c r="M28">
-        <v>4.634</v>
+        <v>4.63853</v>
       </c>
       <c r="N28">
-        <v>-74.156</v>
+        <v>-74.15404</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
@@ -5758,10 +5758,10 @@
         <v>1</v>
       </c>
       <c r="M29">
-        <v>4.626</v>
+        <v>4.63012</v>
       </c>
       <c r="N29">
-        <v>-74.145</v>
+        <v>-74.13848</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
@@ -5802,10 +5802,10 @@
         <v>1</v>
       </c>
       <c r="M30">
-        <v>4.631</v>
+        <v>4.63539</v>
       </c>
       <c r="N30">
-        <v>-74.16</v>
+        <v>-74.15971</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
@@ -5846,10 +5846,10 @@
         <v>1</v>
       </c>
       <c r="M31">
-        <v>4.638</v>
+        <v>4.64272</v>
       </c>
       <c r="N31">
-        <v>-74.15</v>
+        <v>-74.14555</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
@@ -5890,10 +5890,10 @@
         <v>1</v>
       </c>
       <c r="M32">
-        <v>4.627</v>
+        <v>4.63117</v>
       </c>
       <c r="N32">
-        <v>-74.148</v>
+        <v>-74.14273</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -5934,10 +5934,10 @@
         <v>1</v>
       </c>
       <c r="M33">
-        <v>4.6285</v>
+        <v>4.63275</v>
       </c>
       <c r="N33">
-        <v>-74.153</v>
+        <v>-74.1498</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -5978,10 +5978,10 @@
         <v>1</v>
       </c>
       <c r="M34">
-        <v>4.6125</v>
+        <v>4.61597</v>
       </c>
       <c r="N34">
-        <v>-74.155</v>
+        <v>-74.15265</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -6022,10 +6022,10 @@
         <v>1</v>
       </c>
       <c r="M35">
-        <v>4.646</v>
+        <v>4.6511</v>
       </c>
       <c r="N35">
-        <v>-74.145</v>
+        <v>-74.13846</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -6066,10 +6066,10 @@
         <v>1</v>
       </c>
       <c r="M36">
-        <v>4.63</v>
+        <v>4.63434</v>
       </c>
       <c r="N36">
-        <v>-74.1575</v>
+        <v>-74.15617</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
@@ -6110,10 +6110,10 @@
         <v>1</v>
       </c>
       <c r="M37">
-        <v>4.6215</v>
+        <v>4.6254</v>
       </c>
       <c r="N37">
-        <v>-74.149</v>
+        <v>-74.14415</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -6154,10 +6154,10 @@
         <v>1</v>
       </c>
       <c r="M38">
-        <v>4.617</v>
+        <v>4.62072</v>
       </c>
       <c r="N38">
-        <v>-74.17</v>
+        <v>-74.17388</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -6198,10 +6198,10 @@
         <v>1</v>
       </c>
       <c r="M39">
-        <v>4.634</v>
+        <v>4.63854</v>
       </c>
       <c r="N39">
-        <v>-74.1595</v>
+        <v>-74.159</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -6242,10 +6242,10 @@
         <v>1</v>
       </c>
       <c r="M40">
-        <v>4.62</v>
+        <v>4.62383</v>
       </c>
       <c r="N40">
-        <v>-74.152</v>
+        <v>-74.1484</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -6286,10 +6286,10 @@
         <v>1</v>
       </c>
       <c r="M41">
-        <v>4.624</v>
+        <v>4.62802</v>
       </c>
       <c r="N41">
-        <v>-74.144</v>
+        <v>-74.13707</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -6330,10 +6330,10 @@
         <v>1</v>
       </c>
       <c r="M42">
-        <v>4.631</v>
+        <v>4.63535</v>
       </c>
       <c r="N42">
-        <v>-74.137</v>
+        <v>-74.12716</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -6374,10 +6374,10 @@
         <v>1</v>
       </c>
       <c r="M43">
-        <v>4.613</v>
+        <v>4.61648</v>
       </c>
       <c r="N43">
-        <v>-74.15</v>
+        <v>-74.14558</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
@@ -6418,10 +6418,10 @@
         <v>1</v>
       </c>
       <c r="M44">
-        <v>4.619</v>
+        <v>4.6228</v>
       </c>
       <c r="N44">
-        <v>-74.159</v>
+        <v>-74.15831</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -6462,10 +6462,10 @@
         <v>1</v>
       </c>
       <c r="M45">
-        <v>4.632</v>
+        <v>4.63641</v>
       </c>
       <c r="N45">
-        <v>-74.142</v>
+        <v>-74.13423</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
@@ -6506,10 +6506,10 @@
         <v>1</v>
       </c>
       <c r="M46">
-        <v>4.645</v>
+        <v>4.65005</v>
       </c>
       <c r="N46">
-        <v>-74.145</v>
+        <v>-74.13846</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
@@ -6550,10 +6550,10 @@
         <v>1</v>
       </c>
       <c r="M47">
-        <v>4.6368</v>
+        <v>4.64146</v>
       </c>
       <c r="N47">
-        <v>-74.1522</v>
+        <v>-74.14866</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
@@ -6594,10 +6594,10 @@
         <v>1</v>
       </c>
       <c r="M48">
-        <v>4.64</v>
+        <v>4.64482</v>
       </c>
       <c r="N48">
-        <v>-74.15</v>
+        <v>-74.14554</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
@@ -6638,10 +6638,10 @@
         <v>1</v>
       </c>
       <c r="M49">
-        <v>4.654</v>
+        <v>4.6595</v>
       </c>
       <c r="N49">
-        <v>-74.145</v>
+        <v>-74.13845</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
@@ -6682,10 +6682,10 @@
         <v>1</v>
       </c>
       <c r="M50">
-        <v>4.631</v>
+        <v>4.63539</v>
       </c>
       <c r="N50">
-        <v>-74.163</v>
+        <v>-74.16395</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -6726,10 +6726,10 @@
         <v>1</v>
       </c>
       <c r="M51">
-        <v>4.611</v>
+        <v>4.61442</v>
       </c>
       <c r="N51">
-        <v>-74.173</v>
+        <v>-74.17813</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
@@ -6770,10 +6770,10 @@
         <v>1</v>
       </c>
       <c r="M52">
-        <v>4.62</v>
+        <v>4.62386</v>
       </c>
       <c r="N52">
-        <v>-74.17</v>
+        <v>-74.17388</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
@@ -6814,10 +6814,10 @@
         <v>1</v>
       </c>
       <c r="M53">
-        <v>4.6335</v>
+        <v>4.63799</v>
       </c>
       <c r="N53">
-        <v>-74.1465</v>
+        <v>-74.1406</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
@@ -6858,10 +6858,10 @@
         <v>1</v>
       </c>
       <c r="M54">
-        <v>4.628</v>
+        <v>4.63221</v>
       </c>
       <c r="N54">
-        <v>-74.14</v>
+        <v>-74.13141</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -6902,10 +6902,10 @@
         <v>1</v>
       </c>
       <c r="M55">
-        <v>4.614</v>
+        <v>4.61757</v>
       </c>
       <c r="N55">
-        <v>-74.171</v>
+        <v>-74.1753</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
@@ -6946,10 +6946,10 @@
         <v>1</v>
       </c>
       <c r="M56">
-        <v>4.6352</v>
+        <v>4.63978</v>
       </c>
       <c r="N56">
-        <v>-74.1508</v>
+        <v>-74.14668</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
@@ -6990,10 +6990,10 @@
         <v>1</v>
       </c>
       <c r="M57">
-        <v>4.6365</v>
+        <v>4.64115</v>
       </c>
       <c r="N57">
-        <v>-74.155</v>
+        <v>-74.15262</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
@@ -7034,10 +7034,10 @@
         <v>1</v>
       </c>
       <c r="M58">
-        <v>4.6245</v>
+        <v>4.62857</v>
       </c>
       <c r="N58">
-        <v>-74.16</v>
+        <v>-74.15972</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
@@ -7078,21 +7078,24 @@
         <v>1</v>
       </c>
       <c r="M59">
-        <v>4.6235</v>
+        <v>4.62751</v>
       </c>
       <c r="N59">
-        <v>-74.1565</v>
+        <v>-74.15476</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="C10:C259">
+      <formula1>CAPAS!$B$2:$B$30</formula1>
+    </dataValidation>
     <dataValidation type="list" sqref="C2:C259">
       <formula1>CAPAS!$B$2:$B$30</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -10078,16 +10081,22 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <dataValidations count="2">
+  <dataValidations count="4">
+    <dataValidation type="list" sqref="B10:C378">
+      <formula1>NODOS!$A$2:$A$500</formula1>
+    </dataValidation>
     <dataValidation type="list" sqref="B2:C378">
       <formula1>NODOS!$A$2:$A$500</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="D10:D378">
+      <formula1>INTERACCIONES!$B$2:$B$30</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="D2:D378">
       <formula1>INTERACCIONES!$B$2:$B$30</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -10218,7 +10227,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -10321,6 +10330,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fuentes primarias (oficiales/academicas) para nodos que solo tenian prensa o verificar
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/red-pot-kennedy-visor.xlsx
+++ b/datos/red-pot-kennedy-visor.xlsx
@@ -661,7 +661,7 @@
     <t>¿El parque lineal del río Bogotá logrará restaurar la planicie de inundación frente al cambio climático?</t>
   </si>
   <si>
-    <t>Consejo de Estado, Sección Primera, sentencia del 28 de marzo de 2014 sobre la cuenca del río Bogotá (acción popular; verificar radicado antes de citar); Decreto 555 de 2021, arts. 60 y 62 (sdp.gov.co/sites/default/files/decreto_555_de_2021.pdf)</t>
+    <t>Consejo de Estado, Sección Primera, sentencia del 28 de marzo de 2014 sobre la cuenca del río Bogotá (acción popular, radicado 25000-23-27-000-2001-90479-01); Decreto 555 de 2021, arts. 60 y 62 (sdp.gov.co/sites/default/files/decreto_555_de_2021.pdf)</t>
   </si>
   <si>
     <t>NOD-EEP06</t>
@@ -1078,7 +1078,7 @@
     <t>¿Por qué el POT no regula umbrales acústicos biofísicos para proteger la fauna en la EEP?</t>
   </si>
   <si>
-    <t>Pinilla, M., Pulido, L. D. y Cardona, C. M. (2024). Evaluación económica de servicios del humedal El Burro, Bogotá. Sociedad y Economía, 51, e10812872 (doi.org/10.25100/sye.v0i51.12872) (unas 83 especies de fauna registradas, SDA 2021); Secretaría Distrital de Ambiente, Plan de Manejo Ambiental del humedal El Burro, formulado por el IDEA de la Universidad Nacional (ambientebogota.gov.co/documents/10184/804589/PMA+EL+BURRO.pdf); estado de amenaza de Rallus semiplumbeus: verificar en el listado de especies amenazadas del Ministerio de Ambiente (Resolución 1912 de 2017)</t>
+    <t>Pinilla, M., Pulido, L. D. y Cardona, C. M. (2024). Evaluación económica de servicios del humedal El Burro, Bogotá. Sociedad y Economía, 51, e10812872 (doi.org/10.25100/sye.v0i51.12872) (unas 83 especies de fauna registradas, SDA 2021); Secretaría Distrital de Ambiente, Plan de Manejo Ambiental del humedal El Burro, formulado por el IDEA de la Universidad Nacional (ambientebogota.gov.co/documents/10184/804589/PMA+EL+BURRO.pdf); Rallus semiplumbeus (tingua bogotana) figura como En Peligro (EN) en BirdLife International/UICN y en el Libro Rojo de Aves de Colombia (Renjifo et al., 2016); Ministerio de Ambiente, Resolución 1912 de 2017 (listado de especies silvestres amenazadas)</t>
   </si>
   <si>
     <t>NOD-BIO02</t>
@@ -1243,7 +1243,7 @@
     <t>¿El manejo hidráulico mecanicista de la EAAB sacrifica la complejidad ecológica del humedal?</t>
   </si>
   <si>
-    <t>Secretaría Distrital de Ambiente, Plan de Manejo Ambiental del humedal El Burro, formulado por el IDEA de la Universidad Nacional (ambientebogota.gov.co/documents/10184/804589/PMA+EL+BURRO.pdf) (la EAAB formula los planes de manejo, convenio 021 de 2005); Alcaldía de Bogotá, EAAB elimina conexiones erradas (bogota.gov.co/mi-ciudad/habitat/acueducto-cierra-conexiones-de-agua-que-contaminaban-rios-de-bogota); Plan de Saneamiento y Manejo de Vertimientos (PSMV) de la EAAB (verificar acto administrativo)</t>
+    <t>Secretaría Distrital de Ambiente, Plan de Manejo Ambiental del humedal El Burro, formulado por el IDEA de la Universidad Nacional (ambientebogota.gov.co/documents/10184/804589/PMA+EL+BURRO.pdf) (la EAAB formula los planes de manejo, convenio 021 de 2005); Alcaldía de Bogotá, EAAB elimina conexiones erradas (bogota.gov.co/mi-ciudad/habitat/acueducto-cierra-conexiones-de-agua-que-contaminaban-rios-de-bogota); Plan de Saneamiento y Manejo de Vertimientos (PSMV) de la EAAB, aprobado por la SDA mediante Resolución 3257 de 2007 y modificado por la Resolución 03428 de 2017</t>
   </si>
   <si>
     <t>fa-faucet</t>
@@ -1546,7 +1546,7 @@
     <t>¿La saturación de Banderas deteriora el tiempo y la calidad de vida de los viajeros?</t>
   </si>
   <si>
-    <t>TransMilenio S.A., Estación Banderas, Troncal Américas (verificar documento oficial)</t>
+    <t>TransMilenio S.A., Estación Banderas, Troncal Américas; estadísticas de oferta y demanda del SITP (transmilenio.gov.co)</t>
   </si>
   <si>
     <t>fa-right-left</t>
@@ -1600,7 +1600,7 @@
     <t>¿La red zonal garantiza accesibilidad equitativa a los barrios periféricos?</t>
   </si>
   <si>
-    <t>TransMilenio S.A., rutas zonales y alimentadoras del SITP (verificar documento oficial)</t>
+    <t>TransMilenio S.A., rutas zonales y alimentadoras del SITP; estadísticas de oferta y demanda (transmilenio.gov.co)</t>
   </si>
   <si>
     <t>fa-van-shuttle</t>
@@ -1792,7 +1792,7 @@
     <t>¿La sentencia se traduce en acciones concretas en el borde de Kennedy?</t>
   </si>
   <si>
-    <t>Consejo de Estado, Sección Primera, sentencia del 28 de marzo de 2014 sobre la cuenca del río Bogotá (acción popular; verificar radicado antes de citar)</t>
+    <t>Consejo de Estado, Sección Primera, sentencia del 28 de marzo de 2014 sobre la cuenca del río Bogotá (acción popular, radicado 25000-23-27-000-2001-90479-01)</t>
   </si>
   <si>
     <t>fa-gavel</t>
@@ -1819,7 +1819,7 @@
     <t>¿La amenaza se refleja en restricciones efectivas o solo en mapas?</t>
   </si>
   <si>
-    <t>Decreto 555 de 2021, art. 18 (amenaza por inundación) y art. 105 (amenaza por inundación en suelo urbano) (sdp.gov.co/sites/default/files/decreto_555_de_2021.pdf); Alcaldía Local de Kennedy (35% del área inundable, redjurista.com, a_jalkennedy_0003_2021); IDIGER: verificar mapas de amenaza</t>
+    <t>Decreto 555 de 2021, art. 18 (amenaza por inundación) y art. 105 (amenaza por inundación en suelo urbano) (sdp.gov.co/sites/default/files/decreto_555_de_2021.pdf); Alcaldía Local de Kennedy (35% del área inundable, redjurista.com, a_jalkennedy_0003_2021); IDIGER, Inundaciones en Bogotá: causas y zonas de riesgo (idiger.gov.co/escenarios-de-riesgo/inundacion/en-bogota); Secretaría Distrital de Salud, ASIS Localidad Kennedy 2024 (saludata.saludcapital.gov.co)</t>
   </si>
   <si>
     <t>fa-house-flood-water</t>
@@ -2005,7 +2005,7 @@
     <t>¿Mientras persistan las conexiones erradas, la regeneración ecológica es posible?</t>
   </si>
   <si>
-    <t>Alcaldía de Bogotá, EAAB, Plan de Identificación y Corrección de Conexiones Erradas (bogota.gov.co/mi-ciudad/habitat/acueducto-cierra-conexiones-de-agua-que-contaminaban-rios-de-bogota); EAAB, PSMV (verificar acto administrativo)</t>
+    <t>Alcaldía de Bogotá, EAAB, Plan de Identificación y Corrección de Conexiones Erradas (bogota.gov.co/mi-ciudad/habitat/acueducto-cierra-conexiones-de-agua-que-contaminaban-rios-de-bogota); EAAB, PSMV: SDA, Resolución 3257 de 2007 y Resolución 03428 de 2017</t>
   </si>
   <si>
     <t>fa-biohazard</t>

</xml_diff>